<commit_message>
Add "Upland" option to peat awcs_wetland_class dropdown
A peat test hole can be sited in an upland (non-wetland) area, which has no
AWCS wetland class. Add "Upland" as a selectable value:

- create_peat_template.R: append "Upland" to the awcs_wetland_class dropdown
  (a non-wetland option, not an AWCS class) and note it in the README sheet;
  regenerate peat_data_entry.xlsx.
- 02_qaqc.Rmd: accept "Upland" in valid_classes so it is not flagged
  UNRECOGNISED_WETLAND_CLASS.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/templates/peat_data_entry.xlsx
+++ b/inst/templates/peat_data_entry.xlsx
@@ -163,7 +163,7 @@
     <t xml:space="preserve">plots — header fields</t>
   </si>
   <si>
-    <t xml:space="preserve">project_id / plot_id: identifiers (plot_id is the primary key for the test hole) | crew: field crew names | awcs_wetland_class: AWCS class-and-form from the dropdown (Bog / Fen / Marsh / Swamp / Shallow Open Water variants) | utm_zone: UTM zone 11N or 12N (NAD83) | gps_easting / gps_northing: UTM coordinates in the zone above | elevation_m: ground elevation above sea level (m) | dominant_bryophyte: dominant surface bryophyte (scientific name, e.g. Sphagnum fuscum) | water_table_depth_m: depth to water table (m) below ground surface — one value per test hole | ph: peat / pore-water pH — one value per test hole | conductivity_us_cm: electrical conductivity (uS/cm) — one value per test hole | remarks: free-text notes from the field-sheet footer</t>
+    <t xml:space="preserve">project_id / plot_id: identifiers (plot_id is the primary key for the test hole) | crew: field crew names | awcs_wetland_class: AWCS class-and-form from the dropdown (Bog / Fen / Marsh / Swamp / Shallow Open Water variants, or Upland for a non-wetland test hole) | utm_zone: UTM zone 11N or 12N (NAD83) | gps_easting / gps_northing: UTM coordinates in the zone above | elevation_m: ground elevation above sea level (m) | dominant_bryophyte: dominant surface bryophyte (scientific name, e.g. Sphagnum fuscum) | water_table_depth_m: depth to water table (m) below ground surface — one value per test hole | ph: peat / pore-water pH — one value per test hole | conductivity_us_cm: electrical conductivity (uS/cm) — one value per test hole | remarks: free-text notes from the field-sheet footer</t>
   </si>
   <si>
     <t xml:space="preserve">horizons — peat profile</t>
@@ -743,7 +743,7 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
-            <xm:f>"Wooded Bog,Shrubby Bog,Wooded Fen,Shrubby Fen,Graminoid Fen,Graminoid Marsh,Submersed/Floating Shallow Open Water,Coniferous Wooded Swamp,Mixedwood Wooded Swamp,Deciduous Wooded Swamp,Shrubby Swamp"</xm:f>
+            <xm:f>"Wooded Bog,Shrubby Bog,Wooded Fen,Shrubby Fen,Graminoid Fen,Graminoid Marsh,Submersed/Floating Shallow Open Water,Coniferous Wooded Swamp,Mixedwood Wooded Swamp,Deciduous Wooded Swamp,Shrubby Swamp,Upland"</xm:f>
           </x14:formula1>
           <xm:sqref>E4:E1003</xm:sqref>
         </x14:dataValidation>

</xml_diff>